<commit_message>
Publish spreadsheet update via web page
</commit_message>
<xml_diff>
--- a/DGS LIST.xlsx
+++ b/DGS LIST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://feisst-my.sharepoint.com/personal/chisora_h_npe-tech_co_nz/Documents/Documents/NPE Tools/DG-Map/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="885" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0C3B1E4-595C-406C-A73B-581CD4205C02}"/>
+  <xr:revisionPtr revIDLastSave="896" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{103FB33C-17CF-464B-83A4-53A71B44D5C7}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-11235" windowWidth="29040" windowHeight="15720" xr2:uid="{F977427A-6EEF-496F-83AC-E1A3F4E254D6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="972" uniqueCount="647">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="998" uniqueCount="665">
   <si>
     <t>Job</t>
   </si>
@@ -1980,6 +1980,60 @@
   </si>
   <si>
     <t>1688 Turakina Valley Road, Marton</t>
+  </si>
+  <si>
+    <t>1087566 - 00070520 - DG Label</t>
+  </si>
+  <si>
+    <t>26 Kent Street, Carterton</t>
+  </si>
+  <si>
+    <t>1087565 - 00063216 - DG Label</t>
+  </si>
+  <si>
+    <t>245 Millricks Line, Linton</t>
+  </si>
+  <si>
+    <t>1087563 - 00065474 - DG Label</t>
+  </si>
+  <si>
+    <t>11 The Oaks, Awapuni</t>
+  </si>
+  <si>
+    <t>1087561 - 00051746 - DG Label</t>
+  </si>
+  <si>
+    <t>25 Weka Street, Pohangina</t>
+  </si>
+  <si>
+    <t>1087623 - 00071450 - DG Label</t>
+  </si>
+  <si>
+    <t>1087622 - 00068633 - DG Label</t>
+  </si>
+  <si>
+    <t>1087621 - 00065427 - DG Label</t>
+  </si>
+  <si>
+    <t>1087620 - 00015005 - DG Label</t>
+  </si>
+  <si>
+    <t>1087619 - 00060420 - DG Label</t>
+  </si>
+  <si>
+    <t>286 Hewitts Road, Linton</t>
+  </si>
+  <si>
+    <t>25 Montgomery Terrace</t>
+  </si>
+  <si>
+    <t>25 Elmira Avenue, Hokowhitu</t>
+  </si>
+  <si>
+    <t>94 Amberley Avenue, Highbury</t>
+  </si>
+  <si>
+    <t>11 Tūere Place, Hokowhitu</t>
   </si>
 </sst>
 </file>
@@ -2352,7 +2406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6218D334-F914-43C7-B5ED-119730E8C2C7}">
-  <dimension ref="A1:C324"/>
+  <dimension ref="A1:C333"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="46" bestFit="1" customWidth="1"/>
@@ -5924,6 +5978,102 @@
         <v>211</v>
       </c>
     </row>
+    <row r="325" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A325" t="s">
+        <v>647</v>
+      </c>
+      <c r="B325" t="s">
+        <v>648</v>
+      </c>
+      <c r="C325" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="326" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A326" t="s">
+        <v>649</v>
+      </c>
+      <c r="B326" t="s">
+        <v>650</v>
+      </c>
+      <c r="C326" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="327" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A327" t="s">
+        <v>651</v>
+      </c>
+      <c r="B327" t="s">
+        <v>652</v>
+      </c>
+      <c r="C327" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="328" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A328" t="s">
+        <v>653</v>
+      </c>
+      <c r="B328" t="s">
+        <v>654</v>
+      </c>
+      <c r="C328" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="329" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A329" t="s">
+        <v>655</v>
+      </c>
+      <c r="B329" t="s">
+        <v>660</v>
+      </c>
+      <c r="C329" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="330" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A330" t="s">
+        <v>656</v>
+      </c>
+      <c r="B330" t="s">
+        <v>661</v>
+      </c>
+      <c r="C330" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="331" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A331" t="s">
+        <v>657</v>
+      </c>
+      <c r="B331" t="s">
+        <v>662</v>
+      </c>
+      <c r="C331" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="332" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A332" t="s">
+        <v>658</v>
+      </c>
+      <c r="B332" t="s">
+        <v>663</v>
+      </c>
+      <c r="C332" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="333" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A333" t="s">
+        <v>659</v>
+      </c>
+      <c r="B333" t="s">
+        <v>664</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>